<commit_message>
Add validation V1/V2 data, sweep scripts, and reference PDFs
Bundles the working-tree state ahead of Pages redeploy: V1/V2
validation projects (DEM tifs, shapefiles, results xlsx, Receivers/
Source zips), analyse/run/sweep scripts under validation/, v2 call
JSON dumps, Bies & Hansen transformer reference, V136-40 wind
turbine spec, and web/LICENSE.
</commit_message>
<xml_diff>
--- a/validation/V1/source level.xlsx
+++ b/validation/V1/source level.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RyanMcKay\OneDrive - Resonate Consultants\Documents\Code\20260427 BEESTY WF attempt\validation\V1\Source levels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RyanMcKay\OneDrive - Resonate Consultants\Documents\Code\20260427 BEESTY WF attempt\validation\V1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D52823E-E79E-42E3-B08E-5366F6DDF520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7CA5D06-971F-43B6-8D20-8D1AB2A8D68E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3570" windowWidth="21810" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>